<commit_message>
Expanded Dataset and prompt template update
</commit_message>
<xml_diff>
--- a/backend/data/Dataset.xlsx
+++ b/backend/data/Dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donno/Local Storage/FYP/ELEC4848/backend/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KC007\Desktop\Test Space\Python\4848\ELEC4848\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55402D8-D972-2D47-8698-2DFAD7400CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396C2E79-964A-49F8-9305-E4AE36F09161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="16560" windowHeight="18580" xr2:uid="{9EFF6F0D-C710-EF47-A58A-AC8F2FE2F277}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="10545" xr2:uid="{9EFF6F0D-C710-EF47-A58A-AC8F2FE2F277}"/>
   </bookViews>
   <sheets>
     <sheet name="Attractions" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="518">
   <si>
     <t>id</t>
   </si>
@@ -245,9 +245,6 @@
     <t>&gt;500</t>
   </si>
   <si>
-    <t>Romantic, Insta-Worthy, Scenic, Local Favorites</t>
-  </si>
-  <si>
     <t>ayld002</t>
   </si>
   <si>
@@ -266,24 +263,12 @@
     <t>22.4673801, 113.9841334</t>
   </si>
   <si>
-    <t>Hidden, Chill</t>
-  </si>
-  <si>
     <t>ayld004</t>
   </si>
   <si>
-    <t>Nam Sang Wai Cable Ferry</t>
-  </si>
-  <si>
-    <t>Tourist Friendly, Chill, Local Favorites, Hidden</t>
-  </si>
-  <si>
     <t>22.453904, 114.034803</t>
   </si>
   <si>
-    <t>The only manual ferry in hong kong, recommended for cyclists</t>
-  </si>
-  <si>
     <t>ayld005</t>
   </si>
   <si>
@@ -296,9 +281,6 @@
     <t>Hiking</t>
   </si>
   <si>
-    <t>Tourist Friendly, Hiking</t>
-  </si>
-  <si>
     <t>ayld006</t>
   </si>
   <si>
@@ -389,27 +371,6 @@
     <t>Family Friendly</t>
   </si>
   <si>
-    <t>Chill, Family Friendly</t>
-  </si>
-  <si>
-    <t>A short walk from MTR Tin Shui Wai Station or the Locwood Light Rail stop brings you to Kingswood Richly Plaza, a cornerstone of daily life for local residents. Unlike the polished, corporate malls typically found in Hong Kong, "Richly" is a maze of small, independently owned stalls and narrow corridors that hum with a distinct, "down-to-earth" energy. It is often described as the "vernacular heart" of the district, offering a stark contrast to the standardized, high-end shopping centers nearby. The plaza is particularly famous as a street food sanctuary. Students and families frequent the first and second floors for affordable snacks, ranging from spicy Sichuan noodles and tofu fa to creative fusion pancakes and Hong Kong-style "cart noodles." Beyond food, the mall is a dense ecosystem of essential services—tucked away in its winding corners, you'll find family clinics, local hair salons, hardware stores, and tiny boutiques selling everything from trendy phone cases to traditional dried goods. For many in Tin Shui Wai, it is more than just a place to shop; it is a vital community hub where the atmosphere is busy, unpretentious, and deeply rooted in the neighborhood's history.</t>
-  </si>
-  <si>
-    <t>Located just to the west of Lau Fau Shan is Ha Pak Nai, widely celebrated as the premier spot in Hong Kong for witnessing the sunset. As the tide recedes, the vast mudflats transform into a natural mirror, reflecting the sky's shifting colors in the shallow, still waters. The landscape is dotted with dense mangroves and weathered oyster beds, forming a unique ecosystem that serves as a sanctuary for rare horseshoe crabs and migratory birds. Looking across Deep Bay, the towering skyscrapers of Shenzhen's Shekou district create a striking contrast against the tranquil coastline. Beyond its natural beauty, the area holds significant historical weight; hidden within the village is a fortified structure dating back to the 1911 Revolution, now a declared monument. Unlike the bustling seafood markets nearby, Ha Pak Nai offers a quiet, reflective atmosphere where the rhythm of the tides and the history of the frontier converge.</t>
-  </si>
-  <si>
-    <t>About 20 minutes by double-decker bus or minibus from MTR Tin Shui Wai Station lies Lau Fau Shan, a seafood town overlooking Shenzhen in Mainland China.After hopping off the bus and wandering down a narrow alleyway, you'll find yourself flanked by a dense row of seafood restaurants and shops selling fresh catches and dried goods. As you emerge from the passage, the view suddenly opens up to the sea. There is a large square where the skyline of Shenzhen's skyscrapers stretches across the water. To your left, you can see the Shenzhen Bay Bridge spanning the waves, which carries travelers by car to the immigration checkpoint in western Shenzhen. The square also features a sculpture of an oyster—the local specialty—making it a perfect "Instagrammable" spot. Along the alley you walked through, you can enjoy ginger-infused sweets and tofu fa (tofu pudding) in addition to seafood, making it a great place for a quick break. It is a town that offers a seafood experience with a vibe quite distinct from the outlying islands or Sai Kung. While the town remains famous for its seafood restaurants today, the local oysters have lost some of their former glory, reportedly due to pollution from the Shenzhen side. Right nearby, vast wetlands stretch across the landscape, and there is an observation deck on the hill of Lau Fau Shan where you can look out over the entire marshy expanse. With Shenzhen situated directly on the opposite bank, you can clearly see the buildings on the other side with the naked eye.</t>
-  </si>
-  <si>
-    <t>Situated in the southern reaches of Yuen Long, Tai Tong Country Park serves as a lush, sprawling escape for city dwellers and is arguably most famous for its seasonal transformation. While Hong Kong is primarily known for its tropical greenery, Tai Tong offers a rare spectacle of "autumn red." Every year between December and January, the Sweet Gum Woods (Liquidambar formosana) along the Tai Tong Shan Road turn various shades of amber, orange, and deep crimson. This phenomenon draws thousands of visitors who come to witness the maple-like foliage, making the narrow road a vibrant, bustling promenade of photographers and families. Beyond the seasonal colors, the park is a gateway to the extensive Tai Lam Country Park, which is the second-largest in Hong Kong. From the Tai Tong entrance, hikers can access the final section (Section 10) of the famous MacLehose Trail, leading toward the tranquil waters of the Tai Lam Chung Reservoir, often referred to as the "Thousand Islands Lake" for its stunning archipelago-like views. The park's infrastructure is well-developed, featuring expansive barbecue pits and picnic sites shaded by towering pine and eucalyptus trees, providing a cool respite even during the humid summer months. The terrain here is accessible yet varied. For those looking for a leisurely stroll, the paved slopes of the Tai Tong Nature Trail offer educational insights into local ecology and geology. For more adventurous explorers, the connecting mountain paths lead to higher elevations, offering sweeping panoramic views of the Yuen Long Plain, the village clusters of Shap Pat Heung, and the distant skyline of Shenzhen across the border. Historically, the area was once a center for forestry and agriculture; today, the nearby Tai Tong Organic Ecopark carries on this legacy, allowing visitors to experience strawberry picking and pony rides, adding a layer of rural charm to the mountainous landscape.</t>
-  </si>
-  <si>
-    <t>Located on the northern edge of Tin Shui Wai in the New Territories, the Hong Kong Wetland Park is a world-class conservation, education, and tourism facility that serves as a vital ecological mitigation area for the surrounding urban development. Spanning over sixty hectares, the park is divided into a large indoor visitor center known as the Wetland Interactive World and an expansive outdoor Wetland Reserve that showcases the diversity of Hong Kong's wetland ecosystems. The journey typically begins in the visitor center, which houses themed exhibition galleries, a 3D cinema, and an indoor swamp adventure play area, providing a high-tech introduction to the importance of wetland conservation before guests venture into the natural habitats. Once outside, the park unfolds into a series of meticulously maintained environments, including the Stream Walk, the Dragonfly Pond, and the Butterfly Garden, where visitors can observe local flora and fauna in their native settings. One of the park's most famous residents is Pui Pui, a salt-water crocodile discovered in the Shan Pui River, who now lives in a dedicated outdoor enclosure designed to mimic her natural habitat. The park is particularly renowned for its Mangrove Boardwalk, a floating path that allows visitors to walk directly over the mudflats to see mudskippers, fiddler crabs, and various mangrove species up close without disturbing the delicate soil. For birdwatchers, the park is a premier destination, especially during the migratory season when thousands of birds stop over in the marshes and freshwater ponds; several three-story bird hides equipped with telescopes are strategically placed around the reserve, offering silent vantage points to observe rare species like the black-faced spoonbill. The landscape provides a striking visual contrast, where the tranquil, horizontal expanse of reeds and water is framed by the vertical forest of high-rise residential towers in Tin Shui Wai, serving as a constant reminder of the delicate balance between urban growth and environmental preservation. Throughout the year, the park hosts various educational workshops and guided tours that highlight the functions of wetlands in water purification and flood control, making it a critical hub for environmental research and community engagement. Whether exploring the Successive Exhibition Galleries or trekking through the Wildside Walk, visitors experience a side of Hong Kong that feels worlds away from the city's neon-lit streets, defined instead by the rhythmic sounds of cicadas and the sight of herons gliding over the water at dusk.</t>
-  </si>
-  <si>
-    <t>If you're looking for a shopping experience that feels a world away from the shiny, cookie-cutter malls in the city center, you've got to check out Tin Sau Bazaar in Tin Shui Wai North, which is basically this open-air grid of about 130 tiny stalls run by the Tung Wah Group of Hospitals to help out the local grassroots community. I stumbled upon it while visiting the nearby Wetland Park, and it has such a raw, neighborhood vibe where you can find everything from super cheap household hardware and stationery to those random little hair salons and garment alteration shops that you don't see much of anymore. It's definitely not fancy—the shops are all housed in these uniform, prefabricated containers lined up in rows—but there's something really authentic about seeing the elderly residents from the surrounding public housing estates chatting with the stall owners, who are often locals themselves trying to make a living with the lower rents. You can pick up daily necessities like dried seafood, fresh eggs, or even some surprisingly good street snacks and halal food for way less than what you'd pay at a chain supermarket, though you have to be prepared for the weather since it's entirely outdoors. I went on a humid afternoon and it was pretty scorching even with the big sun umbrellas they've installed, but when a breeze kicks in or during the cooler months, it's actually a nice place to just wander and see the "real" side of life in the New Territories. It's got a bit of a "dawn market" legacy since it was built to give illegal street hawkers a permanent home, and while it's sometimes a bit quiet on weekdays, it really comes alive during their weekend arts fairs or community events. It might not be a tourist destination in the traditional sense, but if you value social enterprises and want to support a place that actually helps low-income families while finding some hidden gems for a few dollars, it's worth the short Light Rail trip to the Tin Sau stop.</t>
-  </si>
-  <si>
     <t>ryld001</t>
   </si>
   <si>
@@ -524,9 +485,6 @@
     <t>1100-2030</t>
   </si>
   <si>
-    <t>rtwd</t>
-  </si>
-  <si>
     <t>atmd005</t>
   </si>
   <si>
@@ -875,9 +833,6 @@
     <t>Waterfall Bay Park</t>
   </si>
   <si>
-    <t>Ap Liu Street</t>
-  </si>
-  <si>
     <t>Golden Computer Arcade</t>
   </si>
   <si>
@@ -1298,9 +1253,6 @@
     <t>Tourist Friendly, Solo Travelers, Budget</t>
   </si>
   <si>
-    <t>Kwai Chung Plaza is a small, unique shopping venue located outside the Kwai Fong MTR Station. It offers a vibrant and lively atmosphere with hundreds of small, locally-owned shops and kiosks. The plaza is known for its budget-friendly prices and a diverse selection of goods, reminiscent of shopping in Southeast Asian cities. It’s a bustling and welcoming space for shoppers seeking a different experience.</t>
-  </si>
-  <si>
     <t>Kwai Chung Plaza is an indoor shopping venue accessible via the Kwai Fong MTR Station (exit D). The property opened in 1990 and features multiple floors, offering a variety of shops and eateries. There are several floors with food shops and a level selling fresh food such as vegetables and fruits. The plaza can be incredibly crowded, and while some recognizable brand name retailers and casual eateries are present, most of the businesses are locally owned. Taxi availability is assumed, but specific details are not mentioned.</t>
   </si>
   <si>
@@ -1310,11 +1262,6 @@
     <t>Located at the border between the North District of the New Territories in Hong Kong and the Yantian District of Shenzhen in the Mainland, Sha Tau Kok was once a Frontier Closed Area. Following its opening, it has now become a popular destination for day trips, requiring a Closed Area Permit for entry. The first and second phases of Sha Tau Kok Pier have opened, providing transportation options for both individual travelers and day-trip tour groups. The area features spectacular coastlines and unique historical landmarks, such as vintage road signs and the Sun Moon Pavilion. Sha Tau Kok is renowned for its beautiful sea views and cultural history.</t>
   </si>
   <si>
-    <t>Sha Tau Kok Pier is 280 meters long; originally built in the 1960s and later reconstructed in 2004, it is only a 20 to 30-minute boat ride from Kat O and Ap Chau. The pier promenade is a choice for romantic strolls. At the end of the pier, "The Ends of the Earth" paired with a pure white lighthouse offers beautiful scenery. 
-Shun Ping Street features murals on the walls painted by Sha Tau Kok primary school students. At the end of the pier, "The Ends of the Earth" paired with a pure white lighthouse offers beautiful scenery.
-The Old Sha Tau Kok Fire Station is a distinctive landmark of Sha Tau Kok, preserving its former appearance and displaying a 1:1 replica of a century-old hand-drawn fire engine. Chung Ying Street is located at the border and was once a trading center for Hong Kong merchants during the early Reform and Opening-up period; it is now a site of historical witness, featuring a wishing lookout and a garden modeled after the style of old Hong Kong railway stations.</t>
-  </si>
-  <si>
     <t>Apply for a Closed Area Permit to visit Sha Tau Kok. Kaito ferries are available to reach tourist hotspots such as Lai Chi Wo, Kat O, and Ap Chau. Consider avoiding peak hours to avoid crowds. Sha Tau Kok Pier offers a romantic walking route, featuring murals by Sha Tau Kok primary school students on the walls. Enjoy the lighthouse and sea views at "The Ends of the Earth." The Old Sha Tau Kok Fire Station displays a vintage fire engine and is a great spot for photos. Chung Ying Street Garden provides an opportunity to view Chung Ying Street and allows for hanging wishing plaques.</t>
   </si>
   <si>
@@ -1352,13 +1299,307 @@
   </si>
   <si>
     <t>The reservoir is particularly impressive after heavy rainfall, showcasing the dam in full swing. Consider visiting during good weather for optimal photography. Explore Tai Tam Tuk Village for a peaceful experience. You can choose different routes to reach the reservoir depending on your starting point.</t>
+  </si>
+  <si>
+    <t>A diverse location offering nature, food, and a relaxing atmosphere. Visitors can enjoy scenic views, local produce, and a variety of recreational activities.</t>
+  </si>
+  <si>
+    <t>The location features a nursery, observation deck, restrooms, a water filling station, bicycle parking, and phone charging facilities. Bicycle-powered phone chargers are available for visitors. The location offers a scenic walking path along the river, with accessible facilities.</t>
+  </si>
+  <si>
+    <t>Plan your visit during the flowering season or when migratory birds return for optimal scenery. Take a taxi or bus 76K from Sheung Shui MTR to reach the location. Bicycle parking is available on the ground floor. Be mindful of the weather, as rain can impact the atmosphere.</t>
+  </si>
+  <si>
+    <t>Local Favorites, Insta-Worthy, Hidden, Family Friendly, Retrofuturistic</t>
+  </si>
+  <si>
+    <t>Outdoor, Coastal, Natural Beauty, Hiking</t>
+  </si>
+  <si>
+    <t>Tap Mun, an island located north of the Sai Kung West Country Park, is a popular day trip and overnight wild camping location for Hongkongers. It's known for its grassy hilltop, numerous cows, and a mix of heritage, history, geology, and natural beauty. Visitors can enjoy a loop trail, ferry access, and various amenities like restaurants and dried fish.</t>
+  </si>
+  <si>
+    <t>Public toilets, casual eateries and restaurants at the Old Fisherman's Village, dry fish, fishing, a loop trail, a few pavilion rest stops, a New Fisherman's Village with more eateries, rope repelling, a few geological features (Balanced Rock, Tap Mun Cave), and a scenic harbor. The ferry departs from Wong Shek Pier, and the boat ride is approximately 1.5 hours. There are also minibus and bus lines connecting from ferry pier to Tai Po and  Shatin.</t>
+  </si>
+  <si>
+    <t>Pack appropriate clothing and footwear for hiking, bring water and snacks, check the ferry schedule before setting off, and be mindful of the cows and their grazing space. Consider bringing a camera to capture the stunning scenery.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Solo Travelers, Family Friendly</t>
+  </si>
+  <si>
+    <t>The Hong Kong UNESCO Global Geopark offers a unique outdoor experience with stunning volcanic landscapes and hiking opportunities. It's a popular destination for nature lovers and adventure seekers.</t>
+  </si>
+  <si>
+    <t>No specific facilities are mentioned.</t>
+  </si>
+  <si>
+    <t>To visit UNESCO Global Geopark, you should plan for a remote excursion as private vehicles and Ubers are prohibited; the most direct way is taking a red taxi to the East Dam or taking MTR to Diamond Hill (Exit C2) to catch Bus 92 to Sai Kung. Since the area functions as a wilderness with no shops or restaurants, it is essential to bring your own food and water in a backpack, especially if you plan to climb the "big hill" for the best views of the ocean and hexagonal rock formations. For a more structured experience, you can visit the Volcanic Discovery Centre at the Sai Kung bus terminus to join a guided tour or coordinate ferry trips from Ma Liu Shui Pier, though note that these ferries generally only operate on weekends and public holidays. Be mindful that while one review incorrectly places Po Pin Chau in Lantau, it is actually located in Sai Kung, and the trip is best enjoyed on a clear, warm day to fully appreciate the dramatic coastal scenery.</t>
+  </si>
+  <si>
+    <t>Insta-Worthy, Hidden, Couples</t>
+  </si>
+  <si>
+    <t>Green Egg Island is a beautiful and tranquil spot on the Clearwater Bay Peninsula, offering kayaking opportunities and a chance to explore the coastline. It's known for its clear water, rocky terrain, and a history of volunteer efforts to clean up marine waste.  The island is relatively close to Sheung Tsz Wan, offering a scenic drive.  It’s a popular destination for both locals and tourists, with a focus on enjoying the natural beauty and a vibrant underwater ecosystem.</t>
+  </si>
+  <si>
+    <t>Kayaking rentals are available at Sheung Tsz Wan.  There are several trails available, including the Lung Ha Wan Country Trail.  Public transportation is limited.  Speedboats are available.</t>
+  </si>
+  <si>
+    <t>Be aware of tides and currents.  Check the weather forecast before heading out.  Respect the environment and dispose of your trash properly.  Consider bringing waterproof gear.</t>
+  </si>
+  <si>
+    <t>Murray House is a large, ex government official residence originally located in the Central area of Hong Kong. It was once a Government House and later served as an officer's quarters during British rule. The building features a beautiful colonial design and has undergone several renovations and exorcisms, including a second exorcism in 1974. It now houses shops and restaurants and offers views of the bay.</t>
+  </si>
+  <si>
+    <t>The building features outdoor verandahs, commercial spaces, restaurants, and a retail outlet. It also has a pier and a waterfront view.</t>
+  </si>
+  <si>
+    <t>Visit the building if you are interested in Hong Kong's history and heritage. It’s a significant landmark and offers a glimpse into the city's past.</t>
+  </si>
+  <si>
+    <t>Tourist Friendly, Family Friendly, Free</t>
+  </si>
+  <si>
+    <t>This small specialist museum in Stanley, Hong Kong, focuses on the history of the prison system and its impact on the local community. It offers free admission and features exhibits on the history of correctional services, including displays of instruments used for punishment and information about the Vietnamese refugee situation.</t>
+  </si>
+  <si>
+    <t>The museum features 10 small galleries spaced out over two floors. Exhibitions represent over 170 years of history dating from the late Qing Dynasty through the colonial period all the way to the present era of National Security Law. The rooms are curated with photos and images from the past, various artefacts and information related to dealing with pirates in the early days, to prison internments during the Japanese occupation, the Vietnamese refugee situation as well as general prison life at the old Victoria prison. There are mock gallows and prison cells as well.</t>
+  </si>
+  <si>
+    <t>If you're in Stanley and have an interest in local correctional services, this museum offers a unique and informative experience. It's a good place to learn about the history of Hong Kong's prison system and its impact on the community.</t>
+  </si>
+  <si>
+    <t>Waterfall Bay Park is a unique urban escape in the Southern District, offering stunning views of Lamma Island and the sea. It's a popular spot for sunset viewing, photography, and sketching, and is a key highlight along the Island South Trail.  The park is highly recommended, but accessibility can be challenging due to locked stairs and the presence of trash on the mudflats.</t>
+  </si>
+  <si>
+    <t>The park features flat paths, nearby shopping malls and restaurants in Wah Fu Estate, and a small beach area. Nearby amenities include shopping malls and restaurants in Wah Fu Estate.</t>
+  </si>
+  <si>
+    <t>Leave no trace principles are strongly encouraged to preserve this rare city hidden gem. Waterfall Bay Park, located in the Southern District near Wah Fu Estate, is a unique urban escape famous for its "Fu Lam Falls" which cascades directly into the sea against a backdrop of panoramic views featuring Lamma Island and transoceanic container vessels. While the waterfall originated from the Pok Fu Lam Reservoir and may not be as massive as it once was, visitors describe it as surprisingly majestic—especially after heavy rain—though its proximity to a large private residential building creates a striking contrast between nature and high-density urban development. The park is highly recommended as a picturesque spot for sunset viewing, photography, and sketching, and it serves as a key highlight along the Island South Trail connecting Pok Fu Lam to Stanley. Accessibility is generally convenient with flat paths and nearby amenities like shopping malls and restaurants in Wah Fu Estate, though visitors must exercise caution as the direct stairs to the waterfall are often locked, sometimes leading people to climb railings for access. Beyond the natural scenery and a small beach area, the park holds historical intrigue with an abandoned wartime bunker nearby, but reviewers consistently express disappointment regarding the accumulation of trash on the mudflats and strongly urge everyone to practice "leave no trace" principles to preserve this rare city hidden gem.</t>
+  </si>
+  <si>
+    <t>Ap Liu Street Market</t>
+  </si>
+  <si>
+    <t>Sham Shui Po's Ap Liu Street is a bustling flea market and electronic hub, known as "Electronic Street," offering a wide range of bargain goods and collectibles. It's a popular destination for locals and tourists alike, particularly for electronics and vintage items.</t>
+  </si>
+  <si>
+    <t>The street is directly adjacent to MTR Sham Shui Po station Exit A2 and C2. Visitors can easily access the market via these stations.  There are numerous stalls offering electronics, vintage goods, and household items.  The area features specialized sections for SIM cards and mobile accessories.  The street is a pedestrian-only zone.</t>
+  </si>
+  <si>
+    <t>Be prepared to negotiate prices, but be cautious of counterfeit items.  Take your time to explore the stalls and discover hidden treasures.  Walking and wandering is encouraged to fully appreciate the market's atmosphere.</t>
+  </si>
+  <si>
+    <t>rssp001</t>
+  </si>
+  <si>
+    <t>Dragon Centre Food Court</t>
+  </si>
+  <si>
+    <t>Urban, Indoor</t>
+  </si>
+  <si>
+    <t>Golden Computer Arcade is a popular arcade and electronics store in Sham Shui Po, offering a wide selection of tech and gaming equipment. It's a landmark known for its extensive inventory and a unique, sometimes chaotic, atmosphere.</t>
+  </si>
+  <si>
+    <t>The arcade features multiple floors with distinct sections catering to different tech interests. The upper floor specializes in new laptops and components, while the lower floor focuses on internal parts like CPUs and motherboards. The middle floor offers a diverse range of products, including retro gaming and cutting-edge tech. The arcade is located near Pei Ho Street, Fuk Wa Street, and Ap Liu Street, providing ample opportunities for browsing and shopping.</t>
+  </si>
+  <si>
+    <t>Price check everything when shopping at the arcade, as multiple shops offer similar items at different prices. Be prepared for a potentially crowded and busy environment.</t>
+  </si>
+  <si>
+    <t>The Ten Thousand Buddhas Monastery in Sha Tin offers a serene and visually stunning experience, characterized by a challenging but rewarding climb to a hilltop complex with numerous golden Buddha statues. While appreciated for its atmosphere, the climb is demanding and may not be suitable for all fitness levels.</t>
+  </si>
+  <si>
+    <t>The monastery features a main temple with a pagoda, various sculptures, and a staircase leading to a hilltop complex. Visitors can access the monastery via a 10-minute walk from MTR Sha Tin Station (Exit B), navigating a somewhat hidden path near a shopping center and cemetery. The ascent involves over 400 steps lined with golden Buddha statues. The site is open daily from 9:00 AM to 5:30 PM, but photography is prohibited inside the main temple.</t>
+  </si>
+  <si>
+    <t>Plan for a physical workout due to the steep climb. Be aware that the site is primarily accessed on foot. Respect the rules prohibiting photography inside the main temple.</t>
+  </si>
+  <si>
+    <t>Sha Tau Kok has a 280 meter long pier; It is only a 20 to 30-minute boat ride from Kat O and Ap Chau. At the end of the pier, ""The Ends of the Earth"" paired with a pure white lighthouse. Shun Ping Street features murals on the walls painted by Sha Tau Kok primary school students. At the end of the pier, "The Ends of the Earth" paired with a pure white lighthouse offers beautiful scenery. The Old Sha Tau Kok Fire Station is a distinctive landmark of Sha Tau Kok, preserving its former appearance and displaying a 1:1 replica of a century-old hand-drawn fire engine. Chung Ying Street is located at the border and was once a trading center for Hong Kong merchants during the early Reform and Opening-up period; it is now a site of historical witness, featuring a wishing lookout and a garden modeled after the style of old Hong Kong railway stations.</t>
+  </si>
+  <si>
+    <t>Kingswood Richly Plaza is a bustling, no-frills labyrinth in Tin Shui Wai, known for its cheap street food and nostalgic atmosphere. It’s a beloved community hub for residents seeking affordable luxuries.</t>
+  </si>
+  <si>
+    <t>The mall features narrow, claustrophobic corridors and mediocre cleanliness. It offers a wide variety of cheap and cheerful options, including claw machine shops, budget hair salons, and family-run eateries. There is a 'Nerdvana' atmosphere with a 'shoulder-to-shoulder' dining experience.</t>
+  </si>
+  <si>
+    <t>Be prepared for a chaotic and crowded experience. Seek out affordable treasures within the mall's cramped stalls.  Utilize the MTR exit near the mall for easy access to other parts of Tin Shui Wai.</t>
+  </si>
+  <si>
+    <t>Solo Travelers, Elderly Friendly</t>
+  </si>
+  <si>
+    <t>Ha Pak Nai is a popular Hong Kong sunset destination known for its tidal flats that reflect the sky and views of the Shenzhen container port. However, accessing the beach involves a challenging commute, including a 15-minute walk or a 2-hour hike, and is hampered by low-frequency minibus service, large crowds, and narrow roads. The experience is a test of patience due to mosquito issues, muddy terrain, and potential rainy spring conditions.</t>
+  </si>
+  <si>
+    <t>The primary transportation is the No. 33 minibus from Yuen Long or Tin Shui Wai. Access to the beach involves a 15-minute walk from the minibus stop or a 2-hour hike via the Pineapple Hill trail. Drivers should be warned about narrow roads and difficult taxi availability during the return trip.</t>
+  </si>
+  <si>
+    <t>Bring insect repellent and plenty of time if you decide the Instagrammable views are worth the trek. Be prepared for muddy terrain and potential rainy spring conditions.</t>
+  </si>
+  <si>
+    <t>Local Favorites, Solo Travelers</t>
+  </si>
+  <si>
+    <t>Lau Fau Shan is a gritty, authentic Hong Kong village located in the northwestern New Territories, offering a unique experience centered around seafood, oyster farming, and a glimpse into the area's industrial history. While it lacks luxury amenities, it's a popular destination for bargain hunters seeking fresh seafood and unique goods, with a caveat regarding hygiene and a potentially smelly shoreline. It offers stunning views of Shenzhen Bay Bridge and the Shekou skyline, and holds historical significance as a former hotspot for illegal immigration.</t>
+  </si>
+  <si>
+    <t>Reaching the village from Central takes about 90 minutes via MTR and bus. From my perspective, Lau Fau Shan is the ultimate destination for "unfiltered" Hong Kong culture; it is not for those who prioritize cleanliness or a "tourist-ready" presentation, but for anyone who wants to see the raw, industrial beauty of the oyster bays and experience a way of life that feels increasingly rare in the modern city. The village offers a glimpse into the area's industrial history and provides a unique opportunity to experience a less polished, more authentic Hong Kong.</t>
+  </si>
+  <si>
+    <t>Be prepared for a muddy shoreline and potential hygiene concerns. Utilize the MTR feeder bus for transportation. Bring appropriate footwear for navigating the uneven terrain. Consider visiting during the off-season to avoid crowds.</t>
+  </si>
+  <si>
+    <t>Nam Sang Wai</t>
+  </si>
+  <si>
+    <t>Nam Sang Wai is a nature and scenery escape offering a unique view of the Shenzhen skyline and surrounding marshlands. It’s a popular spot for hikers and bird watchers, particularly during the pandemic, and provides a tranquil space for cycling and exercise. The area’s scenery shifts with the seasons, making it a reliable destination for urban Hong Kong visitors seeking a quiet escape.</t>
+  </si>
+  <si>
+    <t>No specific facilities are mentioned in the reviews. The location offers a panoramic view of the Shenzhen skyline and surrounding marshlands.  Cycling and exercise are encouraged.</t>
+  </si>
+  <si>
+    <t>Visit during the shoulder seasons (spring or autumn) for pleasant weather.  Utilize cycling paths and walking trails to explore the area.  Be mindful of the surrounding marshlands and potential wildlife.</t>
+  </si>
+  <si>
+    <t>Tai Tong Country Park is a premier Nature &amp; Scenery destination renowned for its spectacular Sweet Gum Woods, offering scenic trails suitable for all fitness levels. Visitors can choose from leisurely routes starting from the Tai Tong Barbecue Plantation or more adventurous hikes towards Tin Fu Tsai, including a farm stay. Careful timing is crucial due to parking difficulties during the peak 'red leaf' season.</t>
+  </si>
+  <si>
+    <t>The park features clean public toilets and snack kiosks at the Tai Tong Barbecue Plantation. Public transport options include the K66 bus stop and the Yuen Tsuen Ancient Trail, with options for taxi availability. The park offers a scenic walk with a beautiful view of the Sweet Gum Woods.</t>
+  </si>
+  <si>
+    <t>Plan your trip around the 'red leaf' season to maximize your experience. Utilize public transport to avoid parking difficulties. Check the official 'red leaf index' for accurate foliage conditions before heading out.</t>
+  </si>
+  <si>
+    <t>The park offers a standard Visitor Centre ($30 HKD) with accessible pathways, observation towers, and a bird-watching hide.  There are mangrove boardwalks, a wetland discovery centre, and a bird-watching hide.  The main Visitor Centre is undergoing a major enhancement project expected to conclude in late 2026.  MTR exits are not explicitly mentioned, but the park is easily accessible via the Tin Shui Wai MTR station.</t>
+  </si>
+  <si>
+    <t>Visit during the winter months (December-January) for the best reflections of the Bald Cypress trees.  Bring binoculars for birdwatching.  Be prepared for crowds, especially during peak season.  Check the park's website for updates on the enhancement project.</t>
+  </si>
+  <si>
+    <t>The Hong Kong Wetland Park is a 61-hectare sanctuary offering a peaceful, family-friendly escape from the surrounding high-rises. Known for its serene "mirror of the sky" aesthetic, the park features mangrove boardwalks, bird-watching hides, and the famous resident crocodile, Pui Pui. While the outdoor reserves remain open for a $30 entry fee, the visitor center is currently undergoing renovations until late 2026.</t>
+  </si>
+  <si>
+    <t>Tin Sau Bazaar is a vibrant social enterprise market in Tin Shui Wai, offering a unique shopping experience with a focus on affordability and community support. It's a hidden gem known for its diverse stalls, traditional food, and supportive local vendors.</t>
+  </si>
+  <si>
+    <t>The market features four zones: food, daily necessities, services, and cooked snacks. It includes specialized finds like aged Chenpi, authentic Indian curry, and fresh herbal soup ingredients. The layout is divided into four zones, with stalls offering a range of goods and services. Visitors can reach the market by taking LRT route 705 from Tin Shui Wai Station or Bus K73 from Long Ping, or Bus 967/967X from Hong Kong Island.</t>
+  </si>
+  <si>
+    <t>Be prepared for a slightly cluttered and authentic market experience. While some stalls may be a bit old-fashioned, the prices are incredibly affordable and a great way to support local vendors.</t>
+  </si>
+  <si>
+    <t>Go Garden is a 2-hectare alpaca farm in Kam Tin offering a rustic, hands-on experience. While families enjoy interacting with animals, visitors are deterred by the high cost and aging facilities. Entry fees range from $100–$150 per person, with surcharges for feeding and enclosure access. It’s best enjoyed with own snacks and prioritizing animal interaction.</t>
+  </si>
+  <si>
+    <t>Entry fees range from $100–$150 per person. The farm’s outdated infrastructure and pricey tuck shop limit accessibility. There are no specific transit directions provided, but the farm is five-minute walk from Kam Sheung Road MTR station. Visitors are advised to bring their own snacks and prioritize animal interaction over modern amenities.</t>
+  </si>
+  <si>
+    <t>Due to the high cost and aging facilities, consider bringing your own snacks and prioritizing animal interaction.  The farm is best enjoyed with your own snacks and a focus on interacting with the animals.</t>
+  </si>
+  <si>
+    <t>Hong Kong version of Miami, a trending Nature &amp; Scenery destination with stunning waterfront views and a cinematic atmosphere. It's a secluded industrial area with limited facilities, requiring visitors to be self-sufficient.</t>
+  </si>
+  <si>
+    <t>No public toilets, trash cans, or convenience stores are available. Visitors must bring their own food, water, and garbage bags for sustenance and waste disposal.</t>
+  </si>
+  <si>
+    <t>Plan your transport and supplies carefully, as the location is isolated and requires careful planning to avoid being stranded without basic necessities. It is currently inaccessible due to the construction of a bus depot.</t>
+  </si>
+  <si>
+    <t>22.332204, 114.190280</t>
+  </si>
+  <si>
+    <t>22.323837, 114.197860</t>
+  </si>
+  <si>
+    <t>22.307034, 114.226071</t>
+  </si>
+  <si>
+    <t>22.329514, 114.220712</t>
+  </si>
+  <si>
+    <t>22.356277, 114.132864</t>
+  </si>
+  <si>
+    <t>22.358148, 114.127621</t>
+  </si>
+  <si>
+    <t>22.546093959,114.224355423</t>
+  </si>
+  <si>
+    <t>22.506791, 114.108666</t>
+  </si>
+  <si>
+    <t>22.47596, 114.36197</t>
+  </si>
+  <si>
+    <t>22.357161, 114.373003</t>
+  </si>
+  <si>
+    <t>22.362050, 114.371522</t>
+  </si>
+  <si>
+    <t>22.303763, 114.310979</t>
+  </si>
+  <si>
+    <t>22.253560, 114.255455</t>
+  </si>
+  <si>
+    <t>22.244548, 114.221863</t>
+  </si>
+  <si>
+    <t>22.217975, 114.209753</t>
+  </si>
+  <si>
+    <t>22.216338, 114.218025</t>
+  </si>
+  <si>
+    <t>22.250926, 114.134742</t>
+  </si>
+  <si>
+    <t>22.330655, 114.162047</t>
+  </si>
+  <si>
+    <t>22.332070, 114.162047</t>
+  </si>
+  <si>
+    <t>22.388093, 114.184948</t>
+  </si>
+  <si>
+    <t>22.36282, 114.15125</t>
+  </si>
+  <si>
+    <t>22.377391, 114.185382</t>
+  </si>
+  <si>
+    <t>22.391044, 114.252899</t>
+  </si>
+  <si>
+    <t>22.427163, 114.265092</t>
+  </si>
+  <si>
+    <t>22.54591, 114.42853</t>
+  </si>
+  <si>
+    <t>22.472381, 114.232922</t>
+  </si>
+  <si>
+    <t>Kwai Chung Plaza is a small, unique shopping venue located outside the Kwai Fong MTR Station. It offers a vibrant and lively atmosphere with hundreds of small, locally-owned shops and kiosks selling cheap street foods. The plaza is known for its budget-friendly prices and a diverse selection of goods, reminiscent of shopping in Southeast Asian cities. It’s a bustling and welcoming space for shoppers seeking a different experience.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1374,6 +1615,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1399,15 +1646,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1464,7 +1714,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1780,21 +2030,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BCA1562-3E79-344E-9B82-D003F5E54972}">
-  <dimension ref="A1:K120"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L120"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.1640625" customWidth="1"/>
+    <col min="2" max="2" width="21.125" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="19.6640625" customWidth="1"/>
-    <col min="8" max="8" width="28.1640625" customWidth="1"/>
+    <col min="4" max="4" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="19.625" customWidth="1"/>
+    <col min="8" max="8" width="28.125" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
     <col min="10" max="10" width="20.5" customWidth="1"/>
     <col min="11" max="11" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1811,37 +2061,37 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="G1" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="H1" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="I1" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="J1" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="K1" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="B2" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="C2" t="str">
         <f>IF($A2&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A2,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D2" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="E2" t="s">
         <v>47</v>
@@ -1850,178 +2100,178 @@
         <v>61</v>
       </c>
       <c r="G2" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H2" t="s">
         <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
       <c r="J2" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
       <c r="K2" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="B3" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="C3" t="str">
         <f>IF($A3&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A3,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D3" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="E3" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F3" t="s">
-        <v>342</v>
+        <v>327</v>
       </c>
       <c r="G3" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H3" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="I3" t="s">
-        <v>344</v>
+        <v>329</v>
       </c>
       <c r="J3" t="s">
-        <v>345</v>
+        <v>330</v>
       </c>
       <c r="K3" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="B4" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="C4" t="str">
         <f>IF($A4&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A4,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D4" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="E4" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F4" t="s">
         <v>53</v>
       </c>
       <c r="G4" t="s">
-        <v>347</v>
+        <v>332</v>
       </c>
       <c r="H4" t="s">
         <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>348</v>
+        <v>333</v>
       </c>
       <c r="J4" t="s">
-        <v>349</v>
+        <v>334</v>
       </c>
       <c r="K4" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="B5" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="C5" t="str">
         <f>IF($A5&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A5,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D5" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
       <c r="E5" t="s">
         <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>351</v>
+        <v>336</v>
       </c>
       <c r="G5" t="s">
         <v>63</v>
       </c>
       <c r="H5" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="I5" t="s">
-        <v>353</v>
+        <v>338</v>
       </c>
       <c r="J5" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="K5" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="B6" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="C6" t="str">
         <f>IF($A6&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A6,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D6" t="s">
-        <v>290</v>
+        <v>275</v>
       </c>
       <c r="E6" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F6" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="G6" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H6" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="I6" t="s">
-        <v>358</v>
+        <v>343</v>
       </c>
       <c r="J6" t="s">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="K6" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="B7" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
       <c r="C7" t="str">
         <f>IF($A7&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A7,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D7" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="E7" t="s">
         <v>48</v>
@@ -2030,34 +2280,34 @@
         <v>61</v>
       </c>
       <c r="G7" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="H7" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="I7" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
       <c r="J7" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
       <c r="K7" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B8" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="C8" t="str">
         <f>IF($A8&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A8,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D8" t="s">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="E8" t="s">
         <v>50</v>
@@ -2066,34 +2316,34 @@
         <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="H8" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="I8" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="J8" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="K8" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="B9" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="C9" t="str">
         <f>IF($A9&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A9,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D9" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="E9" t="s">
         <v>48</v>
@@ -2102,106 +2352,106 @@
         <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="H9" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="I9" t="s">
-        <v>369</v>
+        <v>354</v>
       </c>
       <c r="J9" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="K9" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="B10" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="C10" t="str">
         <f>IF($A10&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A10,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D10" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="E10" t="s">
         <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="G10" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="H10" t="s">
-        <v>373</v>
+        <v>358</v>
       </c>
       <c r="I10" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="J10" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="K10" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="B11" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="C11" t="str">
         <f>IF($A11&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A11,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Central &amp; Western</v>
       </c>
       <c r="D11" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="E11" t="s">
         <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="G11" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
       <c r="H11" t="s">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="I11" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
       <c r="J11" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="K11" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="B12" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="C12" t="str">
         <f>IF($A12&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A12,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Eastern</v>
       </c>
       <c r="D12" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="E12" t="s">
         <v>51</v>
@@ -2210,34 +2460,34 @@
         <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="H12" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="I12" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
       <c r="J12" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="K12" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="B13" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="C13" t="str">
         <f>IF($A13&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A13,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Eastern</v>
       </c>
       <c r="D13" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="E13" t="s">
         <v>51</v>
@@ -2246,1168 +2496,1474 @@
         <v>61</v>
       </c>
       <c r="G13" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="H13" t="s">
         <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>387</v>
+        <v>372</v>
       </c>
       <c r="J13" t="s">
-        <v>388</v>
+        <v>373</v>
       </c>
       <c r="K13" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="B14" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="C14" t="str">
         <f>IF($A14&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A14,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Eastern</v>
       </c>
       <c r="D14" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="E14" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="F14" t="s">
         <v>61</v>
       </c>
       <c r="G14" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="H14" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="I14" t="s">
-        <v>390</v>
+        <v>375</v>
       </c>
       <c r="J14" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="K14" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="B15" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="C15" t="str">
         <f>IF($A15&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A15,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Eastern</v>
       </c>
       <c r="D15" t="s">
-        <v>298</v>
+        <v>283</v>
       </c>
       <c r="E15" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F15" t="s">
         <v>53</v>
       </c>
       <c r="G15" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="H15" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="I15" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="J15" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="K15" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="C16" t="str">
         <f>IF($A16&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A16,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Eastern</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="B17" t="s">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="C17" t="str">
         <f>IF($A17&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A17,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Islands</v>
       </c>
       <c r="D17" t="s">
-        <v>300</v>
+        <v>285</v>
       </c>
       <c r="E17" t="s">
         <v>50</v>
       </c>
       <c r="F17" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="G17" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H17" t="s">
         <v>62</v>
       </c>
       <c r="I17" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="J17" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="K17" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="B18" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="C18" t="str">
         <f>IF($A18&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A18,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Islands</v>
       </c>
       <c r="D18" t="s">
-        <v>301</v>
+        <v>286</v>
       </c>
       <c r="E18" t="s">
         <v>47</v>
       </c>
       <c r="F18" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="G18" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H18" t="s">
         <v>62</v>
       </c>
       <c r="I18" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
       <c r="J18" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
       <c r="K18" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="B19" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="C19" t="str">
         <f>IF($A19&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A19,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Islands</v>
       </c>
       <c r="D19" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="E19" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="F19" t="s">
         <v>61</v>
       </c>
       <c r="G19" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="H19" t="s">
         <v>62</v>
       </c>
       <c r="I19" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
       <c r="J19" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="K19" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="C20" t="str">
         <f>IF($A20&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A20,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Islands</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="C21" t="str">
         <f>IF($A21&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A21,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Islands</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="B22" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="C22" t="str">
         <f>IF($A22&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A22,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kowloon City</v>
       </c>
       <c r="D22" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="E22" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F22" t="s">
-        <v>393</v>
+        <v>378</v>
       </c>
       <c r="G22" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H22" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="I22" t="s">
-        <v>394</v>
+        <v>379</v>
       </c>
       <c r="J22" t="s">
-        <v>395</v>
+        <v>380</v>
       </c>
       <c r="K22" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="B23" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="C23" t="str">
         <f>IF($A23&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A23,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kowloon City</v>
       </c>
+      <c r="D23" t="s">
+        <v>491</v>
+      </c>
       <c r="E23" t="s">
         <v>48</v>
       </c>
       <c r="F23" t="s">
-        <v>397</v>
+        <v>382</v>
       </c>
       <c r="G23" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H23" t="s">
-        <v>398</v>
+        <v>383</v>
       </c>
       <c r="I23" t="s">
-        <v>399</v>
+        <v>384</v>
       </c>
       <c r="J23" t="s">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="K23" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="B24" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="C24" t="str">
         <f>IF($A24&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A24,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kowloon City</v>
       </c>
+      <c r="D24" t="s">
+        <v>492</v>
+      </c>
       <c r="E24" t="s">
         <v>50</v>
       </c>
       <c r="F24" t="s">
-        <v>342</v>
+        <v>327</v>
       </c>
       <c r="G24" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H24" t="s">
-        <v>402</v>
+        <v>387</v>
       </c>
       <c r="I24" t="s">
-        <v>403</v>
+        <v>388</v>
       </c>
       <c r="J24" t="s">
-        <v>404</v>
+        <v>389</v>
       </c>
       <c r="K24" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="C25" t="str">
         <f>IF($A25&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A25,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kowloon City</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="C26" t="str">
         <f>IF($A26&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A26,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kowloon City</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="B27" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="C27" t="str">
         <f>IF($A27&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A27,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwun Tong</v>
       </c>
+      <c r="D27" t="s">
+        <v>493</v>
+      </c>
       <c r="E27" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F27" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="G27" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H27" t="s">
-        <v>406</v>
+        <v>391</v>
       </c>
       <c r="I27" t="s">
-        <v>407</v>
+        <v>392</v>
       </c>
       <c r="J27" t="s">
-        <v>408</v>
+        <v>393</v>
       </c>
       <c r="K27" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="B28" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="C28" t="str">
         <f>IF($A28&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A28,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwun Tong</v>
       </c>
+      <c r="D28" t="s">
+        <v>494</v>
+      </c>
       <c r="E28" t="s">
         <v>50</v>
       </c>
       <c r="F28" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="G28" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H28" t="s">
-        <v>402</v>
+        <v>387</v>
       </c>
       <c r="I28" t="s">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="J28" t="s">
-        <v>411</v>
+        <v>396</v>
       </c>
       <c r="K28" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="C29" t="str">
         <f>IF($A29&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A29,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwun Tong</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="C30" t="str">
         <f>IF($A30&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A30,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwun Tong</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="C31" t="str">
         <f>IF($A31&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A31,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwun Tong</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
       <c r="B32" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="C32" t="str">
         <f>IF($A32&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A32,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwai Tsing</v>
       </c>
+      <c r="D32" t="s">
+        <v>495</v>
+      </c>
       <c r="E32" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F32" t="s">
-        <v>397</v>
+        <v>382</v>
       </c>
       <c r="G32" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H32" t="s">
-        <v>402</v>
+        <v>387</v>
       </c>
       <c r="I32" t="s">
-        <v>414</v>
+        <v>399</v>
       </c>
       <c r="J32" t="s">
-        <v>415</v>
+        <v>400</v>
       </c>
       <c r="K32" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="B33" t="s">
-        <v>413</v>
+        <v>398</v>
       </c>
       <c r="C33" t="str">
         <f>IF($A33&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A33,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwai Tsing</v>
       </c>
+      <c r="D33" t="s">
+        <v>496</v>
+      </c>
       <c r="E33" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="F33" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="G33" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="H33" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="I33" t="s">
-        <v>419</v>
+        <v>517</v>
       </c>
       <c r="J33" t="s">
-        <v>420</v>
+        <v>404</v>
       </c>
       <c r="K33" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="C34" t="str">
         <f>IF($A34&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A34,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwai Tsing</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="C35" t="str">
         <f>IF($A35&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A35,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwai Tsing</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="C36" t="str">
         <f>IF($A36&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A36,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Kwai Tsing</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="B37" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
       <c r="C37" t="str">
         <f>IF($A37&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A37,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>North</v>
       </c>
+      <c r="D37" t="s">
+        <v>497</v>
+      </c>
       <c r="E37" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F37" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="G37" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H37" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="I37" t="s">
-        <v>422</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>423</v>
+        <v>406</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="K37" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
       <c r="B38" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="C38" t="str">
         <f>IF($A38&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A38,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>North</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D38" t="s">
+        <v>498</v>
+      </c>
+      <c r="E38" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" t="s">
+        <v>61</v>
+      </c>
+      <c r="G38" t="s">
+        <v>297</v>
+      </c>
+      <c r="H38" t="s">
+        <v>62</v>
+      </c>
+      <c r="I38" t="s">
+        <v>420</v>
+      </c>
+      <c r="J38" t="s">
+        <v>421</v>
+      </c>
+      <c r="K38" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="C39" t="str">
         <f>IF($A39&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A39,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>North</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="C40" t="str">
         <f>IF($A40&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A40,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>North</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="C41" t="str">
         <f>IF($A41&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A41,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>North</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C42" t="str">
         <f>IF($A42&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A42,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sai Kung</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D42" t="s">
+        <v>499</v>
+      </c>
+      <c r="E42" t="s">
+        <v>50</v>
+      </c>
+      <c r="F42" t="s">
+        <v>423</v>
+      </c>
+      <c r="G42" t="s">
+        <v>424</v>
+      </c>
+      <c r="H42" t="s">
+        <v>358</v>
+      </c>
+      <c r="I42" t="s">
+        <v>425</v>
+      </c>
+      <c r="J42" t="s">
+        <v>426</v>
+      </c>
+      <c r="K42" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="B43" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="C43" t="str">
         <f>IF($A43&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A43,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sai Kung</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D43" t="s">
+        <v>500</v>
+      </c>
+      <c r="E43" t="s">
+        <v>307</v>
+      </c>
+      <c r="F43" t="s">
+        <v>428</v>
+      </c>
+      <c r="G43" t="s">
+        <v>297</v>
+      </c>
+      <c r="H43" t="s">
+        <v>429</v>
+      </c>
+      <c r="I43" t="s">
+        <v>430</v>
+      </c>
+      <c r="J43" t="s">
+        <v>431</v>
+      </c>
+      <c r="K43" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="B44" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
       <c r="C44" t="str">
         <f>IF($A44&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A44,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sai Kung</v>
       </c>
+      <c r="D44" t="s">
+        <v>501</v>
+      </c>
       <c r="E44" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F44" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="G44" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="H44" t="s">
-        <v>398</v>
+        <v>383</v>
       </c>
       <c r="I44" t="s">
-        <v>425</v>
+        <v>408</v>
       </c>
       <c r="J44" t="s">
-        <v>426</v>
+        <v>409</v>
       </c>
       <c r="K44" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="B45" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="C45" t="str">
         <f>IF($A45&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A45,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sai Kung</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D45" t="s">
+        <v>502</v>
+      </c>
+      <c r="E45" t="s">
+        <v>50</v>
+      </c>
+      <c r="F45" t="s">
+        <v>433</v>
+      </c>
+      <c r="G45" t="s">
+        <v>297</v>
+      </c>
+      <c r="H45" t="s">
+        <v>358</v>
+      </c>
+      <c r="I45" t="s">
+        <v>434</v>
+      </c>
+      <c r="J45" t="s">
+        <v>435</v>
+      </c>
+      <c r="K45" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="C46" t="str">
         <f>IF($A46&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A46,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sai Kung</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="B47" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="C47" t="str">
         <f>IF($A47&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A47,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Southern</v>
       </c>
+      <c r="D47" t="s">
+        <v>503</v>
+      </c>
       <c r="E47" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F47" t="s">
-        <v>428</v>
+        <v>411</v>
       </c>
       <c r="G47" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="H47" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="I47" t="s">
-        <v>429</v>
+        <v>412</v>
       </c>
       <c r="J47" t="s">
-        <v>430</v>
+        <v>413</v>
       </c>
       <c r="K47" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="B48" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="C48" t="str">
         <f>IF($A48&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A48,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Southern</v>
       </c>
+      <c r="D48" t="s">
+        <v>504</v>
+      </c>
       <c r="E48" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F48" t="s">
-        <v>432</v>
+        <v>415</v>
       </c>
       <c r="G48" t="s">
-        <v>433</v>
+        <v>416</v>
       </c>
       <c r="H48" t="s">
-        <v>402</v>
+        <v>387</v>
       </c>
       <c r="I48" t="s">
-        <v>434</v>
+        <v>417</v>
       </c>
       <c r="J48" t="s">
-        <v>435</v>
+        <v>418</v>
       </c>
       <c r="K48" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="B49" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="C49" t="str">
         <f>IF($A49&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A49,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Southern</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D49" t="s">
+        <v>505</v>
+      </c>
+      <c r="E49" t="s">
+        <v>51</v>
+      </c>
+      <c r="F49" t="s">
+        <v>428</v>
+      </c>
+      <c r="G49" t="s">
+        <v>297</v>
+      </c>
+      <c r="H49" t="s">
+        <v>62</v>
+      </c>
+      <c r="I49" t="s">
+        <v>437</v>
+      </c>
+      <c r="J49" t="s">
+        <v>438</v>
+      </c>
+      <c r="K49" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="B50" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="C50" t="str">
         <f>IF($A50&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A50,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Southern</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D50" t="s">
+        <v>506</v>
+      </c>
+      <c r="E50" t="s">
+        <v>48</v>
+      </c>
+      <c r="F50" t="s">
+        <v>428</v>
+      </c>
+      <c r="G50" t="s">
+        <v>298</v>
+      </c>
+      <c r="H50" t="s">
+        <v>440</v>
+      </c>
+      <c r="I50" t="s">
+        <v>441</v>
+      </c>
+      <c r="J50" t="s">
+        <v>442</v>
+      </c>
+      <c r="K50" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="B51" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="C51" t="str">
         <f>IF($A51&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A51,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Southern</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D51" t="s">
+        <v>507</v>
+      </c>
+      <c r="E51" t="s">
+        <v>307</v>
+      </c>
+      <c r="F51" t="s">
+        <v>54</v>
+      </c>
+      <c r="G51" t="s">
+        <v>332</v>
+      </c>
+      <c r="H51" t="s">
+        <v>109</v>
+      </c>
+      <c r="I51" t="s">
+        <v>444</v>
+      </c>
+      <c r="J51" t="s">
+        <v>445</v>
+      </c>
+      <c r="K51" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="B52" t="s">
-        <v>278</v>
+        <v>447</v>
       </c>
       <c r="C52" t="str">
         <f>IF($A52&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A52,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sham Shui Po</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D52" t="s">
+        <v>508</v>
+      </c>
+      <c r="E52" t="s">
+        <v>51</v>
+      </c>
+      <c r="F52" t="s">
+        <v>61</v>
+      </c>
+      <c r="G52" t="s">
+        <v>367</v>
+      </c>
+      <c r="H52" t="s">
+        <v>62</v>
+      </c>
+      <c r="I52" t="s">
+        <v>448</v>
+      </c>
+      <c r="J52" t="s">
+        <v>449</v>
+      </c>
+      <c r="K52" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="B53" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="C53" t="str">
         <f>IF($A53&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A53,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sham Shui Po</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D53" t="s">
+        <v>509</v>
+      </c>
+      <c r="E53" t="s">
+        <v>51</v>
+      </c>
+      <c r="F53" t="s">
+        <v>61</v>
+      </c>
+      <c r="G53" t="s">
+        <v>453</v>
+      </c>
+      <c r="H53" t="s">
+        <v>62</v>
+      </c>
+      <c r="I53" t="s">
+        <v>454</v>
+      </c>
+      <c r="J53" t="s">
+        <v>455</v>
+      </c>
+      <c r="K53" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="C54" t="str">
         <f>IF($A54&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A54,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sham Shui Po</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="C55" t="str">
         <f>IF($A55&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A55,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sham Shui Po</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="C56" t="str">
         <f>IF($A56&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A56,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sham Shui Po</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="B57" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="C57" t="str">
         <f>IF($A57&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A57,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sha Tin</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D57" t="s">
+        <v>510</v>
+      </c>
+      <c r="E57" t="s">
+        <v>296</v>
+      </c>
+      <c r="F57" t="s">
+        <v>56</v>
+      </c>
+      <c r="G57" t="s">
+        <v>297</v>
+      </c>
+      <c r="H57" t="s">
+        <v>109</v>
+      </c>
+      <c r="I57" t="s">
+        <v>457</v>
+      </c>
+      <c r="J57" t="s">
+        <v>458</v>
+      </c>
+      <c r="K57" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="B58" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="C58" t="str">
         <f>IF($A58&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A58,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sha Tin</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D58" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="B59" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="C59" t="str">
         <f>IF($A59&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A59,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sha Tin</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D59" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="B60" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="C60" t="str">
         <f>IF($A60&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A60,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sha Tin</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D60" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="B61" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="C61" t="str">
         <f>IF($A61&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A61,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Sha Tin</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D61" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>42</v>
       </c>
       <c r="B62" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C62" t="str">
         <f>IF($A62&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A62,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="D62" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E62" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+      <c r="F62" t="s">
+        <v>60</v>
+      </c>
+      <c r="G62" t="s">
+        <v>297</v>
+      </c>
+      <c r="H62" t="s">
+        <v>428</v>
+      </c>
+      <c r="I62" t="s">
+        <v>488</v>
+      </c>
+      <c r="J62" t="s">
+        <v>489</v>
+      </c>
+      <c r="K62" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B63" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C63" t="str">
         <f>IF($A63&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A63,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="D63" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E63" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B64" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C64" t="str">
         <f>IF($A64&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A64,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="D64" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E64" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B65" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C65" t="str">
         <f>IF($A65&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A65,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="D65" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E65" t="s">
         <v>47</v>
       </c>
       <c r="H65" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="C66" t="str">
         <f>IF($A66&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A66,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B67" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C67" t="str">
         <f>IF($A67&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A67,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tai Po</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="D67" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B68" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C68" t="str">
         <f>IF($A68&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A68,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tai Po</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="D68" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="C69" t="str">
         <f>IF($A69&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A69,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tai Po</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="C70" t="str">
         <f>IF($A70&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A70,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tai Po</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="C71" t="str">
         <f>IF($A71&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A71,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tai Po</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="C72" t="str">
         <f>IF($A72&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A72,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tsuen Wan</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="C73" t="str">
         <f>IF($A73&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A73,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tsuen Wan</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="C74" t="str">
         <f>IF($A74&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A74,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tsuen Wan</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="C75" t="str">
         <f>IF($A75&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A75,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tsuen Wan</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="C76" t="str">
         <f>IF($A76&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A76,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tsuen Wan</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="C77" t="str">
         <f>IF($A77&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A77,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wan Chai</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>189</v>
+        <v>175</v>
       </c>
       <c r="C78" t="str">
         <f>IF($A78&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A78,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wan Chai</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="C79" t="str">
         <f>IF($A79&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A79,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wan Chai</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="C80" t="str">
         <f>IF($A80&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A80,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wan Chai</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="C81" t="str">
         <f>IF($A81&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A81,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wan Chai</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="C82" t="str">
         <f>IF($A82&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A82,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wong Tai Sin</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="C83" t="str">
         <f>IF($A83&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A83,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wong Tai Sin</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>224</v>
+        <v>210</v>
       </c>
       <c r="C84" t="str">
         <f>IF($A84&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A84,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wong Tai Sin</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="C85" t="str">
         <f>IF($A85&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A85,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wong Tai Sin</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
       <c r="C86" t="str">
         <f>IF($A86&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A86,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Wong Tai Sin</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>43</v>
       </c>
@@ -3424,341 +3980,458 @@
       <c r="E87" t="s">
         <v>49</v>
       </c>
+      <c r="F87" t="s">
+        <v>61</v>
+      </c>
+      <c r="G87" t="s">
+        <v>367</v>
+      </c>
+      <c r="H87" t="s">
+        <v>61</v>
+      </c>
+      <c r="I87" t="s">
+        <v>461</v>
+      </c>
+      <c r="J87" t="s">
+        <v>462</v>
+      </c>
       <c r="K87" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>68</v>
+      </c>
+      <c r="B88" t="s">
         <v>69</v>
-      </c>
-      <c r="B88" t="s">
-        <v>70</v>
       </c>
       <c r="C88" t="str">
         <f>IF($A88&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A88,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D88" t="s">
+        <v>70</v>
+      </c>
+      <c r="E88" t="s">
+        <v>307</v>
+      </c>
+      <c r="F88" t="s">
+        <v>428</v>
+      </c>
+      <c r="G88" t="s">
+        <v>297</v>
+      </c>
+      <c r="H88" t="s">
+        <v>464</v>
+      </c>
+      <c r="I88" t="s">
+        <v>465</v>
+      </c>
+      <c r="J88" t="s">
+        <v>466</v>
+      </c>
+      <c r="K88" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>71</v>
       </c>
-      <c r="E88" t="s">
-        <v>47</v>
-      </c>
-      <c r="H88" t="s">
-        <v>68</v>
-      </c>
-      <c r="K88" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+      <c r="B89" t="s">
         <v>72</v>
-      </c>
-      <c r="B89" t="s">
-        <v>73</v>
       </c>
       <c r="C89" t="str">
         <f>IF($A89&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A89,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D89" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E89" t="s">
         <v>49</v>
       </c>
+      <c r="F89" t="s">
+        <v>60</v>
+      </c>
+      <c r="G89" t="s">
+        <v>297</v>
+      </c>
       <c r="H89" t="s">
-        <v>75</v>
+        <v>468</v>
+      </c>
+      <c r="I89" t="s">
+        <v>469</v>
+      </c>
+      <c r="J89" t="s">
+        <v>470</v>
       </c>
       <c r="K89" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B90" t="s">
-        <v>77</v>
+        <v>472</v>
       </c>
       <c r="C90" t="str">
         <f>IF($A90&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A90,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D90" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E90" t="s">
         <v>50</v>
       </c>
+      <c r="F90" t="s">
+        <v>307</v>
+      </c>
+      <c r="G90" t="s">
+        <v>60</v>
+      </c>
       <c r="H90" t="s">
-        <v>78</v>
+        <v>297</v>
+      </c>
+      <c r="I90" t="s">
+        <v>109</v>
+      </c>
+      <c r="J90" t="s">
+        <v>473</v>
       </c>
       <c r="K90" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+        <v>474</v>
+      </c>
+      <c r="L90" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B91" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C91" t="str">
         <f>IF($A91&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A91,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D91" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E91" t="s">
         <v>47</v>
       </c>
+      <c r="F91" t="s">
+        <v>307</v>
+      </c>
+      <c r="G91" t="s">
+        <v>54</v>
+      </c>
       <c r="H91" t="s">
-        <v>85</v>
+        <v>332</v>
+      </c>
+      <c r="I91" t="s">
+        <v>109</v>
+      </c>
+      <c r="J91" t="s">
+        <v>476</v>
       </c>
       <c r="K91" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+        <v>477</v>
+      </c>
+      <c r="L91" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B92" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C92" t="str">
         <f>IF($A92&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A92,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D92" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E92" t="s">
-        <v>47</v>
+        <v>307</v>
+      </c>
+      <c r="F92" t="s">
+        <v>428</v>
+      </c>
+      <c r="G92" t="s">
+        <v>297</v>
+      </c>
+      <c r="H92" t="s">
+        <v>109</v>
+      </c>
+      <c r="I92" t="s">
+        <v>481</v>
+      </c>
+      <c r="J92" t="s">
+        <v>479</v>
       </c>
       <c r="K92" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B93" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C93" t="str">
         <f>IF($A93&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A93,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D93" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E93" t="s">
         <v>48</v>
       </c>
+      <c r="F93" t="s">
+        <v>51</v>
+      </c>
+      <c r="G93" t="s">
+        <v>61</v>
+      </c>
+      <c r="H93" t="s">
+        <v>297</v>
+      </c>
+      <c r="I93" t="s">
+        <v>363</v>
+      </c>
+      <c r="J93" t="s">
+        <v>482</v>
+      </c>
       <c r="K93" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+        <v>483</v>
+      </c>
+      <c r="L93" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B94" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C94" t="str">
         <f>IF($A94&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A94,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="D94" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E94" t="s">
         <v>50</v>
       </c>
+      <c r="F94" t="s">
+        <v>61</v>
+      </c>
+      <c r="G94" t="s">
+        <v>297</v>
+      </c>
       <c r="H94" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+      <c r="I94" t="s">
+        <v>485</v>
+      </c>
+      <c r="J94" t="s">
+        <v>486</v>
+      </c>
+      <c r="K94" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C95" t="str">
         <f>IF($A95&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A95,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C96" t="str">
         <f>IF($A96&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A96,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="C97" t="str">
         <f>IF($A97&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A97,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yau Tsim Mong</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="C98" t="str">
         <f>IF($A98&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A98,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yau Tsim Mong</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="C99" t="str">
         <f>IF($A99&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A99,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yau Tsim Mong</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="C100" t="str">
         <f>IF($A100&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A100,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yau Tsim Mong</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="C101" t="str">
         <f>IF($A101&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A101,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yau Tsim Mong</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C102" t="str">
         <f>IF($A102&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A102,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C103" t="str">
         <f>IF($A103&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A103,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C104" t="str">
         <f>IF($A104&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A104,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C105" t="str">
         <f>IF($A105&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A105,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C106" t="str">
         <f>IF($A106&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A106,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C107" t="str">
         <f>IF($A107&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A107,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C108" t="str">
         <f>IF($A108&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A108,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C109" t="str">
         <f>IF($A109&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A109,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C110" t="str">
         <f>IF($A110&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A110,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C111" t="str">
         <f>IF($A111&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A111,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C112" t="str">
         <f>IF($A112&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A112,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="113" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C113" t="str">
         <f>IF($A113&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A113,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="114" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C114" t="str">
         <f>IF($A114&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A114,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="115" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C115" t="str">
         <f>IF($A115&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A115,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="116" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="116" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C116" t="str">
         <f>IF($A116&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A116,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="117" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="117" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C117" t="str">
         <f>IF($A117&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A117,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="118" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="118" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C118" t="str">
         <f>IF($A118&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A118,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="119" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C119" t="str">
         <f>IF($A119&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A119,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="120" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="120" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C120" t="str">
         <f>IF($A120&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT($A120,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
@@ -3809,17 +4482,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4651DCB9-6907-D741-96BC-AD60469A8BFE}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.875" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3833,19 +4506,19 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="F1" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="G1" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="H1" t="s">
         <v>4</v>
       </c>
       <c r="I1" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="J1" t="s">
         <v>5</v>
@@ -3854,442 +4527,445 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C2" t="str">
         <f>IF(A2&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A2,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="E2" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="F2" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="G2" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="H2" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="I2" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="K2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="C3" t="str">
         <f>IF(A3&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A3,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="E3" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="F3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H3" t="s">
+        <v>121</v>
+      </c>
+      <c r="I3" t="s">
+        <v>125</v>
+      </c>
+      <c r="K3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>126</v>
       </c>
-      <c r="G3" t="s">
-        <v>137</v>
-      </c>
-      <c r="H3" t="s">
-        <v>134</v>
-      </c>
-      <c r="I3" t="s">
-        <v>138</v>
-      </c>
-      <c r="K3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>139</v>
-      </c>
-      <c r="B4" t="s">
-        <v>152</v>
       </c>
       <c r="C4" t="str">
         <f>IF(A4&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A4,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Yuen Long</v>
       </c>
       <c r="E4" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="G4" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="H4" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="I4" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="K4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="C5" t="str">
         <f>IF(A5&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A5,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="E5" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="F5" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="G5" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="H5" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="I5" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="K5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="C6" t="str">
         <f>IF(A6&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A6,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="E6" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="G6" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="H6" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="I6" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="K6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="C7" t="str">
         <f>IF(A7&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A7,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v>Tuen Mun</v>
       </c>
       <c r="E7" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="G7" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="H7" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="I7" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="K7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>451</v>
+      </c>
+      <c r="B8" t="s">
+        <v>452</v>
       </c>
       <c r="C8" t="str">
         <f>IF(A8&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A8,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
-        <v>Tsuen Wan</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>Sham Shui Po</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C9" t="str">
         <f>IF(A9&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A9,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C10" t="str">
         <f>IF(A10&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A10,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C11" t="str">
         <f>IF(A11&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A11,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C12" t="str">
         <f>IF(A12&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A12,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C13" t="str">
         <f>IF(A13&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A13,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C14" t="str">
         <f>IF(A14&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A14,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C15" t="str">
         <f>IF(A15&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A15,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C16" t="str">
         <f>IF(A16&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A16,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" t="str">
         <f>IF(A17&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A17,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" t="str">
         <f>IF(A18&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A18,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C19" t="str">
         <f>IF(A19&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A19,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C20" t="str">
         <f>IF(A20&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A20,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C21" t="str">
         <f>IF(A21&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A21,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="22" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C22" t="str">
         <f>IF(A22&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A22,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C23" t="str">
         <f>IF(A23&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A23,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="24" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C24" t="str">
         <f>IF(A24&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A24,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C25" t="str">
         <f>IF(A25&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A25,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C26" t="str">
         <f>IF(A26&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A26,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C27" t="str">
         <f>IF(A27&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A27,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C28" t="str">
         <f>IF(A28&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A28,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C29" t="str">
         <f>IF(A29&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A29,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C30" t="str">
         <f>IF(A30&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A30,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C31" t="str">
         <f>IF(A31&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A31,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C32" t="str">
         <f>IF(A32&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A32,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" t="str">
         <f>IF(A33&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A33,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f>IF(A34&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A34,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
         <f>IF(A35&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A35,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36" t="str">
         <f>IF(A36&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A36,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" t="str">
         <f>IF(A37&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A37,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C38" t="str">
         <f>IF(A38&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A38,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C39" t="str">
         <f>IF(A39&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A39,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C40" t="str">
         <f>IF(A40&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A40,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41" t="str">
         <f>IF(A41&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A41,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42" t="str">
         <f>IF(A42&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A42,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43" t="str">
         <f>IF(A43&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A43,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C44" t="str">
         <f>IF(A44&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A44,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45" t="str">
         <f>IF(A45&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A45,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46" t="str">
         <f>IF(A46&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A46,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C47" t="str">
         <f>IF(A47&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A47,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48" t="str">
         <f>IF(A48&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A48,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C49" t="str">
         <f>IF(A49&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A49,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C50" t="str">
         <f>IF(A50&lt;&gt;"", _xlfn.IFNA(VLOOKUP(RIGHT(LEFT(A50,4),3),'District LookUp Table'!$A$2:$B$19,2,FALSE), "NOT FOUND"), "")</f>
         <v/>
@@ -4311,12 +4987,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8AED754-AC12-BD44-80EC-D17D8DEA7029}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4324,7 +5000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -4332,7 +5008,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -4340,7 +5016,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -4348,7 +5024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -4356,7 +5032,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -4364,7 +5040,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -4372,7 +5048,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -4380,7 +5056,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -4388,7 +5064,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -4396,7 +5072,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -4404,7 +5080,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -4412,7 +5088,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4420,7 +5096,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -4428,7 +5104,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -4436,7 +5112,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -4444,15 +5120,15 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B17" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -4460,7 +5136,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -4476,15 +5152,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA0276EE-1648-024A-B5FF-0F186E065FBF}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>46</v>
       </c>
@@ -4492,16 +5168,16 @@
         <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="D1" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="E1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -4509,7 +5185,7 @@
         <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="D2" t="s">
         <v>62</v>
@@ -4518,7 +5194,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -4526,16 +5202,16 @@
         <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -4546,13 +5222,13 @@
         <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="E4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -4563,13 +5239,13 @@
         <v>64</v>
       </c>
       <c r="D5" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="E5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -4577,40 +5253,40 @@
         <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="D6" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="B7" t="s">
         <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="D7" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="B8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>61</v>
       </c>

</xml_diff>